<commit_message>
Cierre 2026-10-20 15:13 — "Master único en Costos, corrección de catálogo y limpieza"
</commit_message>
<xml_diff>
--- a/Presupuestos/Obras/Obra005/data/pedir_precios_005.xlsx
+++ b/Presupuestos/Obras/Obra005/data/pedir_precios_005.xlsx
@@ -8,14 +8,27 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Dropbox\Analisis_de_costos_y_Presupuestacion\Presupuestos\Obras\Obra005\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5B4DAA96-D8CD-44BF-AC6B-7727D000DDED}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E5B541CD-C532-445B-B486-ABB8BB940A47}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Datos" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="0"/>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
@@ -208,11 +221,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -515,15 +529,16 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:C22"/>
+  <dimension ref="A1:D22"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="8.88671875" style="1"/>
     <col min="2" max="2" width="45.88671875" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="8.88671875" style="1"/>
+    <col min="4" max="4" width="8.88671875" style="2"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -534,7 +549,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
         <v>3</v>
       </c>
@@ -544,8 +559,12 @@
       <c r="C2" s="1" t="s">
         <v>5</v>
       </c>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="D2" s="2">
+        <f>1333.33333333333/0.62</f>
+        <v>2150.5376344086021</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A3" s="1" t="s">
         <v>6</v>
       </c>
@@ -555,8 +574,12 @@
       <c r="C3" s="1" t="s">
         <v>5</v>
       </c>
-    </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="D3" s="2">
+        <f>59000/6/2/3</f>
+        <v>1638.8888888888889</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A4" s="1" t="s">
         <v>8</v>
       </c>
@@ -566,8 +589,11 @@
       <c r="C4" s="1" t="s">
         <v>5</v>
       </c>
-    </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="D4" s="2">
+        <v>6000</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A5" s="1" t="s">
         <v>10</v>
       </c>
@@ -577,8 +603,11 @@
       <c r="C5" s="1" t="s">
         <v>5</v>
       </c>
-    </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="D5" s="2">
+        <v>8000</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A6" s="1" t="s">
         <v>12</v>
       </c>
@@ -589,7 +618,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A7" s="1" t="s">
         <v>15</v>
       </c>
@@ -600,7 +629,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A8" s="1" t="s">
         <v>18</v>
       </c>
@@ -610,8 +639,12 @@
       <c r="C8" s="1" t="s">
         <v>5</v>
       </c>
-    </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="D8" s="2">
+        <f>8000/25</f>
+        <v>320</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A9" s="1" t="s">
         <v>20</v>
       </c>
@@ -621,8 +654,11 @@
       <c r="C9" s="1" t="s">
         <v>22</v>
       </c>
-    </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="D9" s="2">
+        <v>40000</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A10" s="1" t="s">
         <v>23</v>
       </c>
@@ -632,8 +668,11 @@
       <c r="C10" s="1" t="s">
         <v>22</v>
       </c>
-    </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="D10" s="2">
+        <v>80000</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A11" s="1" t="s">
         <v>25</v>
       </c>
@@ -643,8 +682,11 @@
       <c r="C11" s="1" t="s">
         <v>27</v>
       </c>
-    </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="D11" s="2">
+        <v>240</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A12" s="1" t="s">
         <v>28</v>
       </c>
@@ -654,8 +696,11 @@
       <c r="C12" s="1" t="s">
         <v>5</v>
       </c>
-    </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="D12" s="2">
+        <v>7000</v>
+      </c>
+    </row>
+    <row r="13" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A13" s="1" t="s">
         <v>30</v>
       </c>
@@ -665,8 +710,11 @@
       <c r="C13" s="1" t="s">
         <v>14</v>
       </c>
-    </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="D13" s="2">
+        <v>20000</v>
+      </c>
+    </row>
+    <row r="14" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A14" s="1" t="s">
         <v>32</v>
       </c>
@@ -676,8 +724,11 @@
       <c r="C14" s="1" t="s">
         <v>22</v>
       </c>
-    </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="D14" s="2">
+        <v>85000</v>
+      </c>
+    </row>
+    <row r="15" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A15" s="1" t="s">
         <v>34</v>
       </c>
@@ -687,8 +738,11 @@
       <c r="C15" s="1" t="s">
         <v>22</v>
       </c>
-    </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="D15" s="2">
+        <v>80000</v>
+      </c>
+    </row>
+    <row r="16" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A16" s="1" t="s">
         <v>36</v>
       </c>
@@ -698,8 +752,11 @@
       <c r="C16" s="1" t="s">
         <v>5</v>
       </c>
-    </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="D16" s="2">
+        <v>2400</v>
+      </c>
+    </row>
+    <row r="17" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A17" s="1" t="s">
         <v>38</v>
       </c>
@@ -709,8 +766,11 @@
       <c r="C17" s="1" t="s">
         <v>14</v>
       </c>
-    </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="D17" s="2">
+        <v>8900</v>
+      </c>
+    </row>
+    <row r="18" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A18" s="1" t="s">
         <v>40</v>
       </c>
@@ -721,7 +781,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A19" s="1" t="s">
         <v>42</v>
       </c>
@@ -732,7 +792,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="20" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A20" s="1" t="s">
         <v>44</v>
       </c>
@@ -743,7 +803,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="21" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A21" s="1" t="s">
         <v>47</v>
       </c>
@@ -754,7 +814,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="22" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A22" s="1" t="s">
         <v>49</v>
       </c>

</xml_diff>